<commit_message>
samples_test: remove two real buyer rows and author names from the Coretax fixture
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F1YLqZTGvqrkJ3dLGb5C7j
</commit_message>
<xml_diff>
--- a/samples_test/Coretax_Faktur_Template_v1.6.1_SAMPLE.xlsx
+++ b/samples_test/Coretax_Faktur_Template_v1.6.1_SAMPLE.xlsx
@@ -938,7 +938,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R7"/>
+  <dimension ref="A1:R5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="16.08984375" bestFit="1" customWidth="1" style="49" min="2" max="2"/>
@@ -1070,275 +1070,137 @@
       </c>
     </row>
     <row r="4" ht="15.5" customHeight="1" s="49">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="n">
-        <v>46252</v>
-      </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>18/08/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>04</t>
         </is>
       </c>
-      <c r="E4" s="9" t="n"/>
-      <c r="F4" s="9" t="n"/>
-      <c r="G4" s="9" t="n"/>
-      <c r="H4" s="9" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>1100 - AMI - INV - 08 - 26</t>
         </is>
       </c>
-      <c r="I4" s="9" t="n"/>
-      <c r="J4" s="11" t="inlineStr">
-        <is>
-          <t>1000000000213431000000</t>
-        </is>
-      </c>
-      <c r="K4" s="1" t="inlineStr">
-        <is>
-          <t>3275011808820025</t>
-        </is>
-      </c>
-      <c r="L4" s="15" t="inlineStr">
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>1000000000000000000000</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>3200000000000001</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
         <is>
           <t>TIN</t>
         </is>
       </c>
-      <c r="M4" s="9" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>IDN</t>
         </is>
       </c>
-      <c r="N4" s="9" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="O4" s="9" t="inlineStr">
-        <is>
-          <t>SUMANTRI</t>
-        </is>
-      </c>
-      <c r="P4" s="9" t="inlineStr">
-        <is>
-          <t>KP. RAWA AREN NO. 08, RT. 006, RW. 012, KEL. AREN JAYA KEC. BEKASI TIMUR, KOTA BEKASI JAWA BARAT</t>
-        </is>
-      </c>
-      <c r="Q4" s="10" t="n"/>
-      <c r="R4" s="41" t="inlineStr">
-        <is>
-          <t>3275011808820025000000</t>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>BUDI SANTOSO</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>JL CONTOH NO 1, JAKARTA</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>3200000000000001000000</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15.5" customHeight="1" s="49">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="n">
-        <v>46252</v>
-      </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>18/08/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>04</t>
         </is>
       </c>
-      <c r="E5" s="9" t="n"/>
-      <c r="F5" s="9" t="n"/>
-      <c r="G5" s="9" t="n"/>
-      <c r="H5" s="9" t="inlineStr">
-        <is>
-          <t>1102 - AMI - INV - 08 - 26</t>
-        </is>
-      </c>
-      <c r="I5" s="9" t="n"/>
-      <c r="J5" s="11" t="inlineStr">
-        <is>
-          <t>1000000000213431000000</t>
-        </is>
-      </c>
-      <c r="K5" s="1" t="inlineStr">
-        <is>
-          <t>3302040705750003</t>
-        </is>
-      </c>
-      <c r="L5" s="15" t="inlineStr">
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>1101 - AMI - INV - 08 - 26</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>1000000000000000000000</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>1000000000000002</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
         <is>
           <t>TIN</t>
         </is>
       </c>
-      <c r="M5" s="9" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>IDN</t>
         </is>
       </c>
-      <c r="N5" s="9" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="O5" s="9" t="inlineStr">
-        <is>
-          <t>DARIM</t>
-        </is>
-      </c>
-      <c r="P5" s="9" t="inlineStr">
-        <is>
-          <t>KP. KAUM TENGAH RT. 002 RW. 001, RT. 000, RW. 000 KEL. SIMPANGAN KEC. CIKARANG UTARA KAB. BEKASI JAWA BARAT</t>
-        </is>
-      </c>
-      <c r="Q5" s="10" t="n"/>
-      <c r="R5" s="38" t="inlineStr">
-        <is>
-          <t>3302040705750003000000</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="15.5" customHeight="1" s="49">
-      <c r="A6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>18/08/2026</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>04</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>1100 - AMI - INV - 08 - 26</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>1000000000000000000000</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>3200000000000001</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>TIN</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>IDN</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>BUDI SANTOSO</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>JL CONTOH NO 1, JAKARTA</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>3200000000000001000000</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="15.5" customHeight="1" s="49">
-      <c r="A7" t="n">
-        <v>2</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>18/08/2026</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>04</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>1101 - AMI - INV - 08 - 26</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>1000000000000000000000</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>1000000000000002</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>TIN</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>IDN</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>CV KARYA MANDIRI</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>JL CONTOH NO 2, BEKASI</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr">
+      <c r="R5" t="inlineStr">
         <is>
           <t>1000000000000002000000</t>
         </is>
       </c>
     </row>
+    <row r="6" ht="15.5" customHeight="1" s="49"/>
+    <row r="7" ht="15.5" customHeight="1" s="49"/>
     <row r="8" ht="15.5" customHeight="1" s="49"/>
     <row r="9" ht="15.5" customHeight="1" s="49"/>
     <row r="10" ht="15.5" customHeight="1" s="49"/>

</xml_diff>